<commit_message>
chore: quitar el resaltado de duplicados del Market Analyzer
La hoja traia tres reglas de formato condicional "duplicateValues",
una de ellas sobre B7:B215, la columna de cargos. Pintan texto rojo
sobre fondo rosado, asi que cualquier cargo con el mismo nombre en dos
unidades funcionales salia marcado en el informe del cliente.

Son de cuando se edito la plantilla buscando cargos repetidos, no del
diseño.
</commit_message>
<xml_diff>
--- a/templates/informe-cortesia.xlsx
+++ b/templates/informe-cortesia.xlsx
@@ -17835,15 +17835,6 @@
     <mergeCell ref="B4:H4"/>
     <mergeCell ref="B5:H5"/>
   </mergeCells>
-  <conditionalFormatting sqref="A4">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B7:B215">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B1:C1 A5 B216:C1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
-  </conditionalFormatting>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="landscape" verticalDpi="0" r:id="rId1"/>
   <drawing r:id="rId2"/>

</xml_diff>